<commit_message>
mettre à jour le fichier PRESENCE.xlsx
</commit_message>
<xml_diff>
--- a/PRESENCE.xlsx
+++ b/PRESENCE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tfmcmoc-my.sharepoint.com/personal/engoy_tfm_cmoc_com/Documents/Desktop/ML COURS/LABO - UMK 2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="8_{9598413A-F8DF-4ACC-BF25-917F51D1E76A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2E03DC7-8319-4886-84CF-F94CB185D2AA}"/>
+  <xr:revisionPtr revIDLastSave="59" documentId="8_{9598413A-F8DF-4ACC-BF25-917F51D1E76A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA8B5A48-7854-4385-9E87-8320065BE7C6}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="1" activeTab="1" xr2:uid="{A26C44BA-5B72-4681-97BD-10EA4AFFEFEA}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="26">
   <si>
     <t>NDALA TSHIBEMBE EXAUCE</t>
   </si>
@@ -70,9 +70,6 @@
   </si>
   <si>
     <t>NOM COMPLET</t>
-  </si>
-  <si>
-    <t>Num</t>
   </si>
   <si>
     <t>SUJET</t>
@@ -127,7 +124,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -137,7 +134,14 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -158,7 +162,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -166,21 +170,51 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -658,136 +692,149 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFFBAD2C-166D-4ADE-930D-EC268EC159FF}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="69" style="2" customWidth="1"/>
+    <col min="1" max="1" width="5.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.28515625" style="2" customWidth="1"/>
     <col min="5" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="4" t="s">
+    </row>
+    <row r="2" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A2" s="7">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="3" t="s">
+    </row>
+    <row r="3" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A3" s="7">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+      <c r="D3" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A4" s="7">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" s="3" t="s">
+      <c r="C4" s="8" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+      <c r="D4" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A5" s="7">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="3" t="s">
+      <c r="C5" s="8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+      <c r="D5" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="7">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="3" t="s">
+      <c r="C6" s="8" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+      <c r="D6" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="3" t="s">
+      <c r="C7" s="8" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+      <c r="D7" s="9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A8" s="7">
+        <v>7</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" s="3" t="s">
+      <c r="C8" s="8" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
+      <c r="D8" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="7">
+        <v>8</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="3"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="9"/>
+    </row>
+    <row r="10" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="4"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+    </row>
+    <row r="11" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="4"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update Jupyter notebook with data loading section and execution counts
</commit_message>
<xml_diff>
--- a/PRESENCE.xlsx
+++ b/PRESENCE.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tfmcmoc-my.sharepoint.com/personal/engoy_tfm_cmoc_com/Documents/Desktop/ML COURS/LABO - UMK 2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="59" documentId="8_{9598413A-F8DF-4ACC-BF25-917F51D1E76A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA8B5A48-7854-4385-9E87-8320065BE7C6}"/>
+  <xr:revisionPtr revIDLastSave="82" documentId="8_{9598413A-F8DF-4ACC-BF25-917F51D1E76A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{632B567B-0376-42A2-8EE7-8E2661849CB9}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="1" activeTab="1" xr2:uid="{A26C44BA-5B72-4681-97BD-10EA4AFFEFEA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{A26C44BA-5B72-4681-97BD-10EA4AFFEFEA}"/>
   </bookViews>
   <sheets>
-    <sheet name="PRESENCE" sheetId="1" state="hidden" r:id="rId1"/>
+    <sheet name="PRESENCE" sheetId="1" r:id="rId1"/>
     <sheet name="TPE 1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -550,15 +550,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27CFA285-C12F-43C3-8558-560767DA17D3}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29.5703125" customWidth="1"/>
-    <col min="3" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="7" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -571,8 +571,17 @@
       <c r="D1" s="1">
         <v>46323</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="1">
+        <v>46324</v>
+      </c>
+      <c r="F1" s="1">
+        <v>46325</v>
+      </c>
+      <c r="G1" s="1">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -585,8 +594,14 @@
       <c r="D2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -599,8 +614,14 @@
       <c r="D3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -613,8 +634,14 @@
       <c r="D4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -627,8 +654,14 @@
       <c r="D5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -641,8 +674,14 @@
       <c r="D6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -655,8 +694,14 @@
       <c r="D7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -669,8 +714,14 @@
       <c r="D8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -683,9 +734,14 @@
       <c r="D9">
         <v>0</v>
       </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -698,7 +754,7 @@
     <col min="1" max="1" width="5.28515625" style="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="34.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.28515625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="75.28515625" style="2" customWidth="1"/>
     <col min="5" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>

</xml_diff>